<commit_message>
release: establish v1.0.0 baseline
</commit_message>
<xml_diff>
--- a/test_cases/test_case.xlsx
+++ b/test_cases/test_case.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="17680" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="自动化测试用例" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,195 +12,25 @@
     <sheet name="操作类型说明" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="32">
+  <fonts count="26">
     <font>
       <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <family val="3"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <b val="1"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="0"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
       <sz val="11"/>
     </font>
     <font>
@@ -212,16 +42,147 @@
       <name val="宋体"/>
       <charset val="134"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color rgb="FF9C0006"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color theme="0"/>
+      <sz val="11"/>
+    </font>
     <font/>
-    <font>
-      <b val="1"/>
-      <color rgb="FF9C0006"/>
-    </font>
   </fonts>
-  <fills count="39">
+  <fills count="37">
     <fill>
       <patternFill/>
     </fill>
@@ -231,205 +192,210 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.7999511703848384"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="4" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.5999633777886288"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="4" tint="0.599963377788629"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999511703848384"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="5" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.5999633777886288"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="5" tint="0.599963377788629"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.7999511703848384"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="6" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.5999633777886288"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="6" tint="0.599963377788629"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999511703848384"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="7" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.5999633777886288"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="7" tint="0.599963377788629"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.7999511703848384"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="8" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.5999633777886288"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="8" tint="0.599963377788629"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999511703848384"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="9" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.5999633777886288"/>
-        <bgColor indexed="65"/>
+        <fgColor theme="9" tint="0.599963377788629"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.3999755851924192"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -558,31 +524,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="24" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="24" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="24" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="41" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="24" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="42" fontId="6" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
@@ -591,119 +554,122 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="5" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="6" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="7" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="5" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="7" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -728,70 +694,59 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="31" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1"/>
-    <cellStyle name="货币" xfId="2"/>
-    <cellStyle name="百分比" xfId="3"/>
-    <cellStyle name="千位分隔[0]" xfId="4"/>
-    <cellStyle name="货币[0]" xfId="5"/>
-    <cellStyle name="超链接" xfId="6"/>
-    <cellStyle name="已访问的超链接" xfId="7"/>
-    <cellStyle name="注释" xfId="8"/>
-    <cellStyle name="警告文本" xfId="9"/>
-    <cellStyle name="标题" xfId="10"/>
-    <cellStyle name="解释性文本" xfId="11"/>
-    <cellStyle name="标题 1" xfId="12"/>
-    <cellStyle name="标题 2" xfId="13"/>
-    <cellStyle name="标题 3" xfId="14"/>
-    <cellStyle name="标题 4" xfId="15"/>
-    <cellStyle name="输入" xfId="16"/>
-    <cellStyle name="输出" xfId="17"/>
-    <cellStyle name="计算" xfId="18"/>
-    <cellStyle name="检查单元格" xfId="19"/>
-    <cellStyle name="链接单元格" xfId="20"/>
-    <cellStyle name="汇总" xfId="21"/>
-    <cellStyle name="好" xfId="22"/>
-    <cellStyle name="差" xfId="23"/>
-    <cellStyle name="适中" xfId="24"/>
-    <cellStyle name="强调文字颜色 1" xfId="25"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28"/>
-    <cellStyle name="强调文字颜色 2" xfId="29"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32"/>
-    <cellStyle name="强调文字颜色 3" xfId="33"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36"/>
-    <cellStyle name="强调文字颜色 4" xfId="37"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40"/>
-    <cellStyle name="强调文字颜色 5" xfId="41"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44"/>
-    <cellStyle name="强调文字颜色 6" xfId="45"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1075,7 +1030,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -1085,10 +1039,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S123"/>
+  <dimension ref="A1:S130"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="25.81640625" customWidth="1" min="1" max="1"/>
+    <col width="25.8181818181818" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -1103,7 +1057,7 @@
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="14.453125" customWidth="1" min="17" max="17"/>
+    <col width="14.4545454545455" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
@@ -1284,7 +1238,7 @@
           <t>错误账号测试</t>
         </is>
       </c>
-      <c r="Q2" s="23" t="inlineStr">
+      <c r="Q2" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1381,7 +1335,7 @@
           <t>错误密码测试</t>
         </is>
       </c>
-      <c r="Q3" s="23" t="inlineStr">
+      <c r="Q3" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1472,7 +1426,7 @@
           <t>必填校验</t>
         </is>
       </c>
-      <c r="Q4" s="23" t="inlineStr">
+      <c r="Q4" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1564,7 +1518,7 @@
       <c r="O5" t="n">
         <v>3</v>
       </c>
-      <c r="Q5" s="23" t="inlineStr">
+      <c r="Q5" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1657,7 +1611,7 @@
       <c r="O6" t="n">
         <v>3</v>
       </c>
-      <c r="Q6" s="23" t="inlineStr">
+      <c r="Q6" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1743,7 +1697,7 @@
       <c r="O7" t="n">
         <v>3</v>
       </c>
-      <c r="Q7" s="23" t="inlineStr">
+      <c r="Q7" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1841,7 +1795,7 @@
           <t>正常登录流程</t>
         </is>
       </c>
-      <c r="Q8" s="23" t="inlineStr">
+      <c r="Q8" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -1926,7 +1880,7 @@
       <c r="O9" t="n">
         <v>5</v>
       </c>
-      <c r="Q9" s="23" t="inlineStr">
+      <c r="Q9" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2017,7 +1971,7 @@
       <c r="O10" t="n">
         <v>5</v>
       </c>
-      <c r="Q10" s="23" t="inlineStr">
+      <c r="Q10" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2106,7 +2060,7 @@
       <c r="O11" t="n">
         <v>5</v>
       </c>
-      <c r="Q11" s="23" t="inlineStr">
+      <c r="Q11" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2197,7 +2151,7 @@
       <c r="O12" t="n">
         <v>5</v>
       </c>
-      <c r="Q12" s="23" t="inlineStr">
+      <c r="Q12" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2288,7 +2242,7 @@
       <c r="O13" t="n">
         <v>5</v>
       </c>
-      <c r="Q13" s="23" t="inlineStr">
+      <c r="Q13" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2377,7 +2331,7 @@
       <c r="O14" t="n">
         <v>5</v>
       </c>
-      <c r="Q14" s="23" t="inlineStr">
+      <c r="Q14" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2466,7 +2420,7 @@
       <c r="O15" t="n">
         <v>5</v>
       </c>
-      <c r="Q15" s="23" t="inlineStr">
+      <c r="Q15" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2551,7 +2505,7 @@
       <c r="O16" t="n">
         <v>5</v>
       </c>
-      <c r="Q16" s="23" t="inlineStr">
+      <c r="Q16" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2636,7 +2590,7 @@
       <c r="O17" t="n">
         <v>5</v>
       </c>
-      <c r="Q17" s="23" t="inlineStr">
+      <c r="Q17" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2721,7 +2675,7 @@
       <c r="O18" t="n">
         <v>5</v>
       </c>
-      <c r="Q18" s="23" t="inlineStr">
+      <c r="Q18" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2806,7 +2760,7 @@
       <c r="O19" t="n">
         <v>5</v>
       </c>
-      <c r="Q19" s="23" t="inlineStr">
+      <c r="Q19" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2891,7 +2845,7 @@
       <c r="O20" t="n">
         <v>15</v>
       </c>
-      <c r="Q20" s="23" t="inlineStr">
+      <c r="Q20" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -2977,7 +2931,7 @@
       <c r="O21" t="n">
         <v>10</v>
       </c>
-      <c r="Q21" s="23" t="inlineStr">
+      <c r="Q21" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3063,7 +3017,7 @@
       <c r="O22" t="n">
         <v>10</v>
       </c>
-      <c r="Q22" s="23" t="inlineStr">
+      <c r="Q22" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3149,7 +3103,7 @@
       <c r="O23" t="n">
         <v>10</v>
       </c>
-      <c r="Q23" s="23" t="inlineStr">
+      <c r="Q23" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3235,7 +3189,7 @@
       <c r="O24" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="Q24" s="23" t="inlineStr">
+      <c r="Q24" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3321,7 +3275,7 @@
       <c r="O25" t="n">
         <v>10</v>
       </c>
-      <c r="Q25" s="23" t="inlineStr">
+      <c r="Q25" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3407,7 +3361,7 @@
       <c r="O26" t="n">
         <v>10</v>
       </c>
-      <c r="Q26" s="23" t="inlineStr">
+      <c r="Q26" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3493,7 +3447,7 @@
       <c r="O27" t="n">
         <v>5</v>
       </c>
-      <c r="Q27" s="23" t="inlineStr">
+      <c r="Q27" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3583,7 +3537,7 @@
       <c r="O28" t="n">
         <v>5</v>
       </c>
-      <c r="Q28" s="23" t="inlineStr">
+      <c r="Q28" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3669,7 +3623,7 @@
       <c r="O29" t="n">
         <v>5</v>
       </c>
-      <c r="Q29" s="23" t="inlineStr">
+      <c r="Q29" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3760,9 +3714,9 @@
       <c r="O30" t="n">
         <v>10</v>
       </c>
-      <c r="Q30" s="23" t="inlineStr">
-        <is>
-          <t>pass（全量失败后复跑通过，判定为偶发）</t>
+      <c r="Q30" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -3851,7 +3805,7 @@
       <c r="O31" t="n">
         <v>10</v>
       </c>
-      <c r="Q31" s="23" t="inlineStr">
+      <c r="Q31" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -3945,7 +3899,7 @@
       <c r="O32" t="n">
         <v>10</v>
       </c>
-      <c r="Q32" s="23" t="inlineStr">
+      <c r="Q32" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4039,7 +3993,7 @@
       <c r="O33" t="n">
         <v>10</v>
       </c>
-      <c r="Q33" s="23" t="inlineStr">
+      <c r="Q33" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4056,7 +4010,7 @@
       </c>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>TC-CUSTOMER-014</t>
         </is>
@@ -4133,7 +4087,7 @@
       <c r="O34" t="n">
         <v>10</v>
       </c>
-      <c r="Q34" s="23" t="inlineStr">
+      <c r="Q34" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4227,7 +4181,7 @@
       <c r="O35" t="n">
         <v>10</v>
       </c>
-      <c r="Q35" s="23" t="inlineStr">
+      <c r="Q35" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4321,7 +4275,7 @@
       <c r="O36" t="n">
         <v>10</v>
       </c>
-      <c r="Q36" s="23" t="inlineStr">
+      <c r="Q36" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4415,7 +4369,7 @@
       <c r="O37" t="n">
         <v>10</v>
       </c>
-      <c r="Q37" s="23" t="inlineStr">
+      <c r="Q37" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4509,7 +4463,7 @@
       <c r="O38" t="n">
         <v>10</v>
       </c>
-      <c r="Q38" s="23" t="inlineStr">
+      <c r="Q38" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4525,86 +4479,86 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="28" customFormat="1" customHeight="1" s="21">
-      <c r="A39" s="20" t="inlineStr">
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" t="inlineStr">
         <is>
           <t>TC-CUSTOMER-019</t>
         </is>
       </c>
-      <c r="B39" s="21" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>顾客列表</t>
         </is>
       </c>
-      <c r="C39" s="21" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>备注筛选</t>
         </is>
       </c>
-      <c r="D39" s="21" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>验证备注筛选</t>
         </is>
       </c>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F39" s="21" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>已登录并进入顾客列表页</t>
         </is>
       </c>
-      <c r="G39" s="20" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t xml:space="preserve">1.点击其他筛选 2.输入备注'123' 3.点击确定 4.点击详情 5.在历史影像中点击影像右侧备注图标 </t>
         </is>
       </c>
-      <c r="H39" s="21" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>div:text-is('顾客档案'), 0.5, button:has-text('其他筛选'), input[placeholder='备注'], .ant-popover .ant-btn-primary</t>
         </is>
       </c>
-      <c r="I39" s="21" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>click, wait, click, input, click</t>
         </is>
       </c>
-      <c r="J39" s="21" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
-      <c r="M39" s="21" t="inlineStr">
-        <is>
-          <t>咨询单特定</t>
-        </is>
-      </c>
-      <c r="N39" s="21" t="inlineStr">
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>测试</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
         <is>
           <t>text_visible</t>
         </is>
       </c>
-      <c r="O39" s="21" t="n">
+      <c r="O39" t="n">
         <v>20</v>
       </c>
-      <c r="P39" s="21" t="inlineStr">
+      <c r="P39" t="inlineStr">
         <is>
           <t>已根据实际DOM调整：删除'已为'步骤；确定按钮用.ant-popover .ant-btn-primary；备注图标用.ant-image + div .anticon</t>
         </is>
       </c>
-      <c r="Q39" s="23" t="inlineStr">
+      <c r="Q39" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="R39" s="21" t="inlineStr">
+      <c r="R39" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="S39" s="21" t="inlineStr">
+      <c r="S39" t="inlineStr">
         <is>
           <t>B</t>
         </is>
@@ -4685,7 +4639,7 @@
           <t>卡片为自定义结构（非ant-list）；性别图标为图片形式无法文本断言；字段验证：姓名/年龄/手机号/上次检测时间/检测次数/详情</t>
         </is>
       </c>
-      <c r="Q40" s="23" t="inlineStr">
+      <c r="Q40" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4702,7 +4656,7 @@
       </c>
     </row>
     <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>TC-CUSTOMER-021</t>
         </is>
@@ -4770,7 +4724,7 @@
       <c r="O41" t="n">
         <v>5</v>
       </c>
-      <c r="Q41" s="23" t="inlineStr">
+      <c r="Q41" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4857,7 +4811,7 @@
       <c r="O42" t="n">
         <v>10</v>
       </c>
-      <c r="Q42" s="23" t="inlineStr">
+      <c r="Q42" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -4945,7 +4899,7 @@
       <c r="O43" t="n">
         <v>3</v>
       </c>
-      <c r="Q43" s="23" t="inlineStr">
+      <c r="Q43" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5133,7 +5087,7 @@
       <c r="O45" t="n">
         <v>10</v>
       </c>
-      <c r="Q45" s="23" t="inlineStr">
+      <c r="Q45" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5226,7 +5180,7 @@
       <c r="O46" t="n">
         <v>10</v>
       </c>
-      <c r="Q46" s="23" t="inlineStr">
+      <c r="Q46" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5319,7 +5273,7 @@
       <c r="O47" t="n">
         <v>10</v>
       </c>
-      <c r="Q47" s="23" t="inlineStr">
+      <c r="Q47" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5412,7 +5366,7 @@
       <c r="O48" t="n">
         <v>15</v>
       </c>
-      <c r="Q48" s="23" t="inlineStr">
+      <c r="Q48" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5429,7 +5383,7 @@
       </c>
     </row>
     <row r="49" ht="42" customHeight="1">
-      <c r="A49" s="14" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>TC-DETAIL-007</t>
         </is>
@@ -5500,7 +5454,7 @@
       <c r="O49" t="n">
         <v>15</v>
       </c>
-      <c r="Q49" s="23" t="inlineStr">
+      <c r="Q49" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5517,7 +5471,7 @@
       </c>
     </row>
     <row r="50" ht="42" customHeight="1">
-      <c r="A50" s="14" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>TC-DETAIL-008</t>
         </is>
@@ -5588,7 +5542,7 @@
           <t>清空家庭住址后保存</t>
         </is>
       </c>
-      <c r="Q50" s="23" t="inlineStr">
+      <c r="Q50" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5681,7 +5635,7 @@
           <t>家庭住址输入特殊字符后保存</t>
         </is>
       </c>
-      <c r="Q51" s="23" t="inlineStr">
+      <c r="Q51" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5769,9 +5723,9 @@
           <t>家庭住址输入空格后保存</t>
         </is>
       </c>
-      <c r="Q52" s="23" t="inlineStr">
-        <is>
-          <t>pass（全量失败后复跑通过，判定为偶发）</t>
+      <c r="Q52" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -5816,7 +5770,7 @@
           <t>已登录，进入顾客详情页</t>
         </is>
       </c>
-      <c r="G53" s="15" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>1.点击编辑资料
 2.清空手机号
@@ -5856,7 +5810,7 @@
       <c r="O53" t="n">
         <v>3</v>
       </c>
-      <c r="Q53" s="23" t="inlineStr">
+      <c r="Q53" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -5873,7 +5827,7 @@
       </c>
     </row>
     <row r="54" ht="42" customHeight="1">
-      <c r="A54" s="14" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>TC-DETAIL-012</t>
         </is>
@@ -5903,7 +5857,7 @@
           <t>已登录，进入顾客详情页</t>
         </is>
       </c>
-      <c r="G54" s="15" t="inlineStr">
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>1.已登录，进入顾客详情页
 2.点击右侧所有影像中的一个影像的右下角编辑图标
@@ -5935,7 +5889,7 @@
           <t>备注记录中显示最新的提交记录</t>
         </is>
       </c>
-      <c r="M54" s="17" t="inlineStr">
+      <c r="M54" s="14" t="inlineStr">
         <is>
           <t>123</t>
         </is>
@@ -5948,7 +5902,7 @@
       <c r="O54" t="n">
         <v>5</v>
       </c>
-      <c r="Q54" s="23" t="inlineStr">
+      <c r="Q54" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6036,7 +5990,7 @@
           <t>清空备注后保存，备注非必填</t>
         </is>
       </c>
-      <c r="Q55" s="23" t="inlineStr">
+      <c r="Q55" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6129,7 +6083,7 @@
           <t>备注输入特殊字符后保存</t>
         </is>
       </c>
-      <c r="Q56" s="23" t="inlineStr">
+      <c r="Q56" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6212,7 +6166,7 @@
       <c r="O57" t="n">
         <v>10</v>
       </c>
-      <c r="Q57" s="23" t="inlineStr">
+      <c r="Q57" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6308,7 +6262,7 @@
           <t>nav进入顾客列表，影像编辑图标易缺失，因此改为更稳妥的div</t>
         </is>
       </c>
-      <c r="Q58" s="23" t="inlineStr">
+      <c r="Q58" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6394,7 +6348,7 @@
       <c r="O59" t="n">
         <v>15</v>
       </c>
-      <c r="Q59" s="23" t="inlineStr">
+      <c r="Q59" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6411,7 +6365,7 @@
       </c>
     </row>
     <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="14" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>TC-DETAIL-018</t>
         </is>
@@ -6441,7 +6395,7 @@
           <t>已登录并进入顾客列表页</t>
         </is>
       </c>
-      <c r="G60" s="15" t="inlineStr">
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>1.进入顾客详情页
 2.查找有检测记录顾客
@@ -6485,12 +6439,12 @@
       <c r="O60" t="n">
         <v>15</v>
       </c>
-      <c r="P60" s="14" t="inlineStr">
+      <c r="P60" t="inlineStr">
         <is>
           <t>nav改为div,输入注意去掉占位符，否则读取不到</t>
         </is>
       </c>
-      <c r="Q60" s="23" t="inlineStr">
+      <c r="Q60" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6576,7 +6530,7 @@
       <c r="O61" t="n">
         <v>15</v>
       </c>
-      <c r="Q61" s="23" t="inlineStr">
+      <c r="Q61" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6666,7 +6620,7 @@
           <t>标签「自动化标签测试1」需已存在（由 TC-DETAIL-016 生成）</t>
         </is>
       </c>
-      <c r="Q62" s="23" t="inlineStr">
+      <c r="Q62" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6761,7 +6715,7 @@
           <t>需要有历史影像</t>
         </is>
       </c>
-      <c r="Q63" s="23" t="inlineStr">
+      <c r="Q63" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6851,7 +6805,7 @@
       <c r="O64" t="n">
         <v>15</v>
       </c>
-      <c r="Q64" s="23" t="inlineStr">
+      <c r="Q64" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -6941,7 +6895,7 @@
           <t>需要有历史影像</t>
         </is>
       </c>
-      <c r="Q65" s="23" t="inlineStr">
+      <c r="Q65" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7030,7 +6984,7 @@
           <t>需要有历史影像；验证管理/完成按钮来回切换</t>
         </is>
       </c>
-      <c r="Q66" s="23" t="inlineStr">
+      <c r="Q66" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7218,7 +7172,7 @@
       <c r="O68" t="n">
         <v>15</v>
       </c>
-      <c r="Q68" s="23" t="inlineStr">
+      <c r="Q68" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7309,7 +7263,7 @@
       <c r="O69" t="n">
         <v>15</v>
       </c>
-      <c r="Q69" s="23" t="inlineStr">
+      <c r="Q69" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7484,7 +7438,7 @@
           <t>需要有历史影像；管理模式下不选影像直接删除应提示</t>
         </is>
       </c>
-      <c r="Q71" s="23" t="inlineStr">
+      <c r="Q71" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7501,7 +7455,7 @@
       </c>
     </row>
     <row r="72" ht="28" customFormat="1" customHeight="1" s="4">
-      <c r="A72" s="16" t="inlineStr">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>TC-DETAIL-030</t>
         </is>
@@ -7580,7 +7534,7 @@
           <t>需要「咨询单特定」测试用户存在且有历史影像</t>
         </is>
       </c>
-      <c r="Q72" s="23" t="inlineStr">
+      <c r="Q72" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7676,7 +7630,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单；咨询单记录在诊断结果标签页</t>
         </is>
       </c>
-      <c r="Q73" s="23" t="inlineStr">
+      <c r="Q73" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7772,7 +7726,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q74" s="23" t="inlineStr">
+      <c r="Q74" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7868,7 +7822,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q75" s="23" t="inlineStr">
+      <c r="Q75" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -7964,7 +7918,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q76" s="23" t="inlineStr">
+      <c r="Q76" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8059,7 +8013,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q77" s="23" t="inlineStr">
+      <c r="Q77" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8154,7 +8108,7 @@
           <t>需先执行 TC-DETAIL-030 创建咨询单</t>
         </is>
       </c>
-      <c r="Q78" s="23" t="inlineStr">
+      <c r="Q78" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8215,12 +8169,12 @@
       </c>
       <c r="H79" s="4" t="inlineStr">
         <is>
-          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), a:has-text('详情'), 3, [role='tabpanel'] .anticon, [role='tabpanel'] .anticon, 3, textarea, textarea, button:has-text('提 交'), text=自动化删除测试${TIMESTAMP}, .ant-timeline .anticon, 2, text=确定</t>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), a:has-text('详情'), 3, [role='tabpanel'] .anticon, [role='tabpanel'] .anticon, 3, textarea, textarea, button:has-text('提 交'), 3, .ant-timeline :has-text('自动化删除测试${TIMESTAMP}'), .ant-timeline .anticon, 2, text=确定, .ant-modal-close, 2, [role='tabpanel'] .anticon, 3</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>click, wait, verify, input, click, wait, verify, click, wait, verify, click, wait, verify, input, click, verify, click, wait, click</t>
+          <t>click, wait, verify, input, click, wait, verify, click, wait, verify, click, wait, verify, input, click, wait, verify, click, wait, click, click, wait, click, wait</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -8244,14 +8198,14 @@
         </is>
       </c>
       <c r="O79" s="4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="P79" s="4" t="inlineStr">
         <is>
           <t>自包含用例：先新增固定备注再删除，验证点固定无需随测试数据更新</t>
         </is>
       </c>
-      <c r="Q79" s="23" t="inlineStr">
+      <c r="Q79" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8796,7 +8750,7 @@
       <c r="O85" t="n">
         <v>5</v>
       </c>
-      <c r="Q85" s="23" t="inlineStr">
+      <c r="Q85" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8886,7 +8840,7 @@
       <c r="O86" t="n">
         <v>5</v>
       </c>
-      <c r="Q86" s="23" t="inlineStr">
+      <c r="Q86" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -8976,7 +8930,7 @@
       <c r="O87" t="n">
         <v>5</v>
       </c>
-      <c r="Q87" s="23" t="inlineStr">
+      <c r="Q87" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9061,7 +9015,7 @@
       <c r="O88" t="n">
         <v>5</v>
       </c>
-      <c r="Q88" s="23" t="inlineStr">
+      <c r="Q88" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9241,7 +9195,7 @@
       <c r="O90" t="n">
         <v>3</v>
       </c>
-      <c r="Q90" s="23" t="inlineStr">
+      <c r="Q90" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9332,7 +9286,7 @@
       <c r="O91" t="n">
         <v>3</v>
       </c>
-      <c r="Q91" s="23" t="inlineStr">
+      <c r="Q91" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9423,7 +9377,7 @@
       <c r="O92" t="n">
         <v>3</v>
       </c>
-      <c r="Q92" s="23" t="inlineStr">
+      <c r="Q92" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -9514,7 +9468,7 @@
       <c r="O93" t="n">
         <v>3</v>
       </c>
-      <c r="Q93" s="23" t="inlineStr">
+      <c r="Q93" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -11993,7 +11947,7 @@
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="14" t="inlineStr">
+      <c r="A121" t="inlineStr">
         <is>
           <t>TC-IMAGE-032</t>
         </is>
@@ -12075,7 +12029,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q121" s="23" t="inlineStr">
+      <c r="Q121" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -12174,7 +12128,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q122" s="23" t="inlineStr">
+      <c r="Q122" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -12190,7 +12144,7 @@
         </is>
       </c>
     </row>
-    <row r="123">
+    <row r="123" ht="84" customHeight="1">
       <c r="A123" t="inlineStr">
         <is>
           <t>TC-IMAGE-034</t>
@@ -12221,7 +12175,7 @@
           <t>已登录</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr">
+      <c r="G123" s="3" t="inlineStr">
         <is>
           <t>1.进入顾客列表
 2.搜索「咨询单特定」
@@ -12273,7 +12227,7 @@
           <t>需要「咨询单特定」测试用户且有历史影像</t>
         </is>
       </c>
-      <c r="Q123" s="23" t="inlineStr">
+      <c r="Q123" s="15" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
@@ -12284,6 +12238,610 @@
         </is>
       </c>
       <c r="S123" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="112" customHeight="1">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>TC-IMAGE-035</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>影像阅览</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>UI验证</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>中文环境UI验证左侧列表</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>已登录</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>1.进入顾客列表
+2.搜索18279763980
+3.进入详情页
+4.在右侧历史影像下方点击左上角P2的影像进入阅览页
+5.从上向下依次校验左侧列表是否包含：视角回正，光影增强，精确测量，无对比，分屏对比，镜像对比，分屏对比，镜像对比</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), 3, [class*='G6f2']:has-text('P2') .ant-image, 15</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>click, wait, verify, input, click, wait, click, wait, click, wait</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>18279763980</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>'视角回正','光影增强','精确测量','无对比','分屏对比','镜像对比'</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>text_visible</t>
+        </is>
+      </c>
+      <c r="O124" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q124" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="98" customHeight="1">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>TC-IMAGE-036</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>影像阅览</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>UI验证</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>中文环境UI验证诊断图谱数量-AI综合分析</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>已登录</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>1.进入顾客列表
+2.搜索18279763980
+3.进入详情页
+4.在右侧历史影像下方点击左上角P2的影像进入阅览页
+5.点击诊断图谱中的AI综合分析
+6.验证上方的图谱是否包含：冷光，粗纹，毛孔，细纹，凹陷</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), 3, [class*='G6f2']:has-text('P2') .ant-image, 15, text=AI综合分析</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>click, wait, verify, input, click, wait, click, wait, click, wait, click, wait</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>18279763980</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>点击诊断图谱中的AI综合分析后，上方图谱包含冷光，粗纹，毛孔，细纹，凹陷</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>'冷光','粗纹','毛孔','细纹','凹陷'</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>text_visible</t>
+        </is>
+      </c>
+      <c r="O125" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q125" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="126" customHeight="1">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>TC-IMAGE-037</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>影像阅览</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>UI验证</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>中文环境UI验证诊断图谱数量-炎敏</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>已登录</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr">
+        <is>
+          <t>1.进入顾客列表
+2.搜索18279763980
+3.进入详情页
+4.在右侧历史影像下方点击左上角P2的影像进入阅览页
+5.点击诊断图谱中的炎敏
+6.验证上方的图谱是否包含：冷光，紫外线，标准红区，增强红区，红区热力，红血丝，交叉偏振</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), 3, [class*='G6f2']:has-text('P2') .ant-image, 15, text=炎敏, 5</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>click, wait, verify, input, click, wait, click, wait, click, wait, click, wait</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>18279763980</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>点击诊断图谱中的炎敏，上方图谱包含冷光，紫外线，标准红区，增强红区，红区热力，红血丝，交叉偏振</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>'冷光','紫外线','标准红区','增强红区','红区热力','红血丝','交叉偏振'</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>text_visible</t>
+        </is>
+      </c>
+      <c r="O126" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q126" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="126" customHeight="1">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>TC-IMAGE-038</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>影像阅览</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>UI验证</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>中文环境UI验证诊断图谱数量-肤色</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>已登录</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>1.进入顾客列表
+2.搜索18279763980
+3.进入详情页
+4.在右侧历史影像下方点击左上角P2的影像进入阅览页
+5.点击诊断图谱中的肤色
+6.验证上方的图谱是否包含：自然光，冷光，标准棕区，紫外线斑，增强棕区，棕区热力，紫外线</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), 3, [class*='G6f2']:has-text('P2') .ant-image, 15, text=肤色</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>click, wait, verify, input, click, wait, click, wait, click, wait, click, wait</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>18279763980</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>点击诊断图谱中的肤色后，上方图谱包含自然光，冷光，标准棕区，紫外线斑，增强棕区，棕区热力，紫外线</t>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>'自然光','冷光','标准棕区','紫外线斑','增强棕区','棕区热力','紫外线'</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>text_visible</t>
+        </is>
+      </c>
+      <c r="O127" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q127" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="112" customHeight="1">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>TC-IMAGE-039</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>影像阅览</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>UI验证</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>中文环境UI验证诊断图谱数量-肤质</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>已登录</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>1.进入顾客列表
+2.搜索18279763980
+3.进入详情页
+4.在右侧历史影像下方点击左上角P2的影像进入阅览页
+5.点击诊断图谱中的肤质
+6.验证上方的图谱是否包含：自然光，毛孔，皮纹，紫外线</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), 3, [class*='G6f2']:has-text('P2') .ant-image, 15, text=肤质</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>click, wait, verify, input, click, wait, click, wait, click, wait, click, wait</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>18279763980</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t>点击诊断图谱中的肤质后，上方图谱包含自然光，毛孔，皮纹，紫外线</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>'自然光','毛孔','皮纹','紫外线'</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>text_visible</t>
+        </is>
+      </c>
+      <c r="O128" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q128" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="112" customHeight="1">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>TC-IMAGE-040</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>影像阅览</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>UI验证</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>中文环境UI验证诊断图谱数量-衰老</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>已登录</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>1.进入顾客列表
+2.搜索18279763980
+3.进入详情页
+4.在右侧历史影像下方点击左上角P2的影像进入阅览页
+5.点击诊断图谱中的衰老
+6.验证上方的图谱是否包含：自然光，皮纹，细纹，粗纹，平行偏振，灰度，等高线</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), 3, [class*='G6f2']:has-text('P2') .ant-image, 15, text=衰老</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>click, wait, verify, input, click, wait, click, wait, click, wait, click, wait</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>18279763980</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>点击诊断图谱中的衰老后，上方图谱包含自然光，皮纹，细纹，粗纹，平行偏振，灰度，等高线</t>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>'自然光','皮纹','细纹','粗纹','平行偏振','灰度','等高线'</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>text_visible</t>
+        </is>
+      </c>
+      <c r="O129" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q129" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="168" customHeight="1">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>TC-IMAGE-041</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>影像阅览</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>UI验证</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>中文环境UI验证模式图谱</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>已登录</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>1.进入顾客列表
+2.搜索18279763980
+3.进入详情页
+4.在右侧历史影像下方点击左上角P2的影像进入阅览页
+5.点击诊断图谱切换为模式图谱
+6.验证下方的图谱是否包含：冷光，自然光，红血丝，增强红区，标准红区，红区热力，深层棕区，标准棕区，浅层棕区，棕区热力，增强综区，紫外线，紫外线斑，平行偏振，交叉偏振，灰度，等高线，毛孔，皮纹，细纹，粗纹，凹陷</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), 3, [class*='G6f2']:has-text('P2') .ant-image, 15, text=模式图谱, 5</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>click, wait, verify, input, click, wait, click, wait, click, wait, click, wait</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>18279763980</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>点击诊断图谱切换为模式图谱并展开后，下方图谱包含冷光，自然光，红血丝，增强红区，标准红区，红区热力，深层棕区，标准棕区，浅层棕区，棕区热力，增强综区，紫外线，紫外线斑，平行偏振，交叉偏振，灰度，等高线，毛孔，皮纹，细纹，粗纹，凹陷</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>'冷光','自然光','红血丝','增强红区','标准红区','红区热力','深层棕区','标准棕区','浅层棕区','棕区热力','增强棕区','紫外线','紫外线斑','平行偏振','交叉偏振','灰度','等高线','毛孔','皮纹','细纹','粗纹','凹陷'</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>text_visible</t>
+        </is>
+      </c>
+      <c r="O130" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q130" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="S130" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
release: publish case-v1.0.7 Excel baseline
</commit_message>
<xml_diff>
--- a/test_cases/test_case.xlsx
+++ b/test_cases/test_case.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化测试用例" sheetId="1" r:id="R1d26cf0fe6c54d86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R1d6b5d6210934391"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="断言类型说明" sheetId="3" r:id="R9b790e48a22543fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="操作类型说明" sheetId="4" r:id="R8c4899646f454d25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化测试用例" sheetId="1" r:id="R8b72a0662d0a4fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="2" r:id="R342f5bc85af446d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="断言类型说明" sheetId="3" r:id="R27902f0022fd49ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="操作类型说明" sheetId="4" r:id="R1c3dbf06e6d64c8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1681,7 +1681,7 @@
 5.再点击完成</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">div:text-is('顾客档案'), 3, a:has-text('详情'), 共检测, 3, a:text-is('管理'), a:text-is('管理'), a:text-is('完成'), a:text-is('完成'), a:text-is('管理')</x:t>
+    <x:t xml:space="preserve">div:text-is('顾客档案'), 3, a:has-text('详情'), 共检测, 3, div.p-20:has-text('所有历史影像') a:text-is('管理'), div.p-20:has-text('所有历史影像') a:text-is('管理'), a:text-is('完成'), a:text-is('完成'), div.p-20:has-text('所有历史影像') a:text-is('管理')</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">click, wait, verify, find_click, wait, verify, click, verify, click, verify</x:t>
@@ -1716,7 +1716,7 @@
 6.点击删除</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">/customer, 0.5, 共检测1次, a:has-text('管理'), input[type='checkbox'], a:has-text('删除'), .footer-btn-danger, /customer, 0.5</x:t>
+    <x:t xml:space="preserve">/customer, 0.5, 共检测1次, div.p-20:has-text('所有历史影像') a:text-is('管理'), input[type='checkbox'], a:has-text('删除'), .footer-btn-danger, /customer, 0.5</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">nav, wait, find_click, click, click, click, click, nav, wait</x:t>
@@ -1819,7 +1819,7 @@
 7.查看该用户卡片</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">/customer, 0.5, 共检测(?:[2-9]|[1-9]\d+)次, a:has-text('管理'), input[type='checkbox'], a:has-text('删除'), .footer-btn-danger, /customer, 0.5</x:t>
+    <x:t xml:space="preserve">/customer, 0.5, 共检测(?![01]次)\d+次, div.p-20:has-text('所有历史影像') a:text-is('管理'), input[type='checkbox'], a:has-text('删除'), .footer-btn-danger, /customer, 0.5</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">
@@ -1841,11 +1841,11 @@
     <x:t xml:space="preserve">1.进入顾客列表
 2.查找有检测记录顾客
 3.进入详情页
-4.点击管理
+4.点击所有历史影像右侧的管理
 5.点击删除</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">div:text-is('顾客档案'), 3, a:has-text('详情'), 共检测, 3, a:text-is('管理'), a:text-is('管理'), text=删除</x:t>
+    <x:t xml:space="preserve">div:text-is('顾客档案'), 3, a:has-text('详情'), 共检测, 3, div.p-20:has-text('所有历史影像') a:text-is('管理'), div.p-20:has-text('所有历史影像') a:text-is('管理'), text=删除</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">click, wait, verify, find_click, wait, verify, click, click</x:t>
@@ -2932,7 +2932,7 @@
     <x:numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <x:numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </x:numFmts>
-  <x:fonts count="26">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -2956,12 +2956,6 @@
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FFFF0000"/>
-      <x:name val="宋体"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FF9C0006"/>
       <x:name val="宋体"/>
     </x:font>
     <x:font>
@@ -3068,13 +3062,8 @@
       <x:color theme="0"/>
       <x:name val="Calibri"/>
     </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="宋体"/>
-    </x:font>
   </x:fonts>
-  <x:fills count="39">
+  <x:fills count="38">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -3104,11 +3093,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFFF00"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFC7CE"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -3365,28 +3349,31 @@
   </x:borders>
   <x:cellStyleXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <x:xf numFmtId="43" fontId="6" fillId="0" borderId="0">
+    <x:xf numFmtId="43" fontId="5" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="44" fontId="6" fillId="0" borderId="0">
+    <x:xf numFmtId="44" fontId="5" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="9" fontId="6" fillId="0" borderId="0">
+    <x:xf numFmtId="9" fontId="5" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="41" fontId="6" fillId="0" borderId="0">
+    <x:xf numFmtId="41" fontId="5" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="42" fontId="6" fillId="0" borderId="0">
+    <x:xf numFmtId="42" fontId="5" fillId="0" borderId="0">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="2">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="2">
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0">
@@ -3395,37 +3382,37 @@
     <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="3">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="0" borderId="3">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="3">
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="4">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="4">
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+    <x:xf numFmtId="0" fontId="14" fillId="8" borderId="5">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="5">
+    <x:xf numFmtId="0" fontId="15" fillId="9" borderId="6">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="6">
+    <x:xf numFmtId="0" fontId="16" fillId="9" borderId="5">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="5">
+    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="7">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="18" fillId="11" borderId="7">
+    <x:xf numFmtId="0" fontId="18" fillId="0" borderId="8">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="8">
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="9">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="20" fillId="0" borderId="9">
+    <x:xf numFmtId="0" fontId="20" fillId="11" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="21" fillId="12" borderId="0">
@@ -3437,80 +3424,77 @@
     <x:xf numFmtId="0" fontId="23" fillId="14" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="15" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="16" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="17" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="18" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="18" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="19" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="19" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="20" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="21" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="21" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="22" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="22" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="23" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="23" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="24" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="24" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="25" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="25" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="26" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="26" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="27" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="27" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="28" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="28" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="29" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="29" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="30" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="30" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="31" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="31" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="32" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="32" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="33" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="33" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="34" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="34" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="35" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="35" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="36" borderId="0">
+    <x:xf numFmtId="0" fontId="5" fillId="36" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="37" borderId="0">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="24" fillId="38" borderId="0">
+    <x:xf numFmtId="0" fontId="23" fillId="37" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -3534,9 +3518,6 @@
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <x:xf numFmtId="0" fontId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="49">
     <x:cellStyle name="常规" xfId="0"/>
@@ -7659,7 +7640,7 @@
       <x:c r="P67" t="s">
         <x:v>519</x:v>
       </x:c>
-      <x:c r="Q67" t="s">
+      <x:c r="Q67" s="4" t="s">
         <x:v>520</x:v>
       </x:c>
       <x:c r="R67" s="11" t="s">
@@ -7815,7 +7796,7 @@
       <x:c r="O70">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="Q70" t="s">
+      <x:c r="Q70" s="4" t="s">
         <x:v>34</x:v>
       </x:c>
       <x:c r="R70" s="11" t="s">
@@ -9415,8 +9396,8 @@
       <x:c r="P99" t="s">
         <x:v>767</x:v>
       </x:c>
-      <x:c r="Q99" t="str">
-        <x:v>pass</x:v>
+      <x:c r="Q99" s="4" t="s">
+        <x:v>34</x:v>
       </x:c>
       <x:c r="R99" t="s">
         <x:v>345</x:v>

</xml_diff>

<commit_message>
release: validate v1.1.13 for formal publication
</commit_message>
<xml_diff>
--- a/test_cases/test_case.xlsx
+++ b/test_cases/test_case.xlsx
@@ -6057,11 +6057,15 @@
       <c r="G35" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="H35" t="s">
-        <v>268</v>
-      </c>
-      <c r="I35" t="s">
-        <v>269</v>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>/customer, 0.5, button:has-text('其他筛选'), text=45岁以上, .ant-popover .ant-btn-primary, a:has-text('详情')</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>nav, wait, click, click, click, click</t>
+        </is>
       </c>
       <c r="J35" t="s">
         <v>270</v>
@@ -6072,11 +6076,15 @@
       <c r="L35" t="s">
         <v>271</v>
       </c>
-      <c r="M35" t="s">
-        <v>182</v>
-      </c>
-      <c r="N35" t="s">
-        <v>53</v>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>45岁以上</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>age_in_range</t>
+        </is>
       </c>
       <c r="O35">
         <v>10</v>
@@ -9547,11 +9555,15 @@
       <c r="G99" s="11" t="s">
         <v>759</v>
       </c>
-      <c r="H99" s="5" t="s">
-        <v>760</v>
-      </c>
-      <c r="I99" s="5" t="s">
-        <v>761</v>
+      <c r="H99" s="5" t="inlineStr">
+        <is>
+          <t>2561x1398, div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), a:has-text('详情'), 3, [data-layout="column"][data-layout-align="center center"], [data-layout="column"][data-layout-align="center center"], 15, text=正在努力下载资源, text=模型加载中, 1, body, text=视角回正, text=R45°, body, text=R45°, body, text=L45°, body, text=R90°, body, text=L90°, body, text=0°, body, text=光影增强, body, text=分屏对比, 1, body, text=镜像对比, 1, body</t>
+        </is>
+      </c>
+      <c r="I99" s="5" t="inlineStr">
+        <is>
+          <t>set_viewport, click, wait, verify, input, click, wait, verify, click, wait, verify, click, wait, wait_hidden, wait_hidden, wait, vision_compare_step, click, verify, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, wait, vision_compare_step, click, wait, vision_compare_step</t>
+        </is>
       </c>
       <c r="J99" s="5" t="s">
         <v>762</v>

</xml_diff>

<commit_message>
release: publish case-v1.0.9 Excel baseline
</commit_message>
<xml_diff>
--- a/test_cases/test_case.xlsx
+++ b/test_cases/test_case.xlsx
@@ -9557,12 +9557,12 @@
       </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t>2561x1398, div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), a:has-text('详情'), 3, [data-layout="column"][data-layout-align="center center"], [data-layout="column"][data-layout-align="center center"], 15, text=正在努力下载资源, text=模型加载中, 1, body, text=视角回正, text=R45°, body, text=R45°, body, text=L45°, body, text=R90°, body, text=L90°, body, text=0°, body, text=光影增强, body, text=分屏对比, 1, body, text=镜像对比, 1, body</t>
+          <t xml:space="preserve">2561x1398, div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), a:has-text('详情'), 3, [data-layout="column"][data-layout-align="center center"], [data-layout="column"][data-layout-align="center center"], 15, text=正在努力下载资源, text=模型加载中, 1, text=视角回正, text=数据整理中, body, text=视角回正, text=R45°, body, text=R45°, body, text=L45°, body, text=R90°, body, text=L90°, body, text=0°, body, text=光影增强, body, text=分屏对比, 1, body, text=镜像对比, 1, body</t>
         </is>
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>set_viewport, click, wait, verify, input, click, wait, verify, click, wait, verify, click, wait, wait_hidden, wait_hidden, wait, vision_compare_step, click, verify, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, wait, vision_compare_step, click, wait, vision_compare_step</t>
+          <t xml:space="preserve">set_viewport, click, wait, verify, input, click, wait, verify, click, wait, verify, click, wait, wait_hidden, wait_hidden, wait, verify, wait_hidden, vision_compare_step, click, verify, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, wait, vision_compare_step, click, wait, vision_compare_step</t>
         </is>
       </c>
       <c r="J99" s="5" t="s">

</xml_diff>

<commit_message>
release: publish case-v1.0.10 Excel baseline
</commit_message>
<xml_diff>
--- a/test_cases/test_case.xlsx
+++ b/test_cases/test_case.xlsx
@@ -9557,12 +9557,12 @@
       </c>
       <c r="H99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2561x1398, div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), a:has-text('详情'), 3, [data-layout="column"][data-layout-align="center center"], [data-layout="column"][data-layout-align="center center"], 15, text=正在努力下载资源, text=模型加载中, 1, text=视角回正, text=数据整理中, body, text=视角回正, text=R45°, body, text=R45°, body, text=L45°, body, text=R90°, body, text=L90°, body, text=0°, body, text=光影增强, body, text=分屏对比, 1, body, text=镜像对比, 1, body</t>
+          <t xml:space="preserve">2561x1398, div:text-is('顾客档案'), 3, input[placeholder='请输入关键字'], input[placeholder='请输入关键字'], button:has-text('搜 索'), 3, a:has-text('详情'), a:has-text('详情'), 3, [data-layout="column"][data-layout-align="center center"], [data-layout="column"][data-layout-align="center center"], 15, text=正在努力下载资源, text=模型加载中, 1, text=视角回正, :text-matches("正在努力下载资源|模型加载中|数据整理中"):visible, 2, :text-matches("正在努力下载资源|模型加载中|数据整理中"):visible, text=视角回正, body, text=视角回正, text=R45°, body, text=R45°, body, text=L45°, body, text=R90°, body, text=L90°, body, text=0°, body, text=光影增强, body, text=分屏对比, 1, body, text=镜像对比, 1, body</t>
         </is>
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">set_viewport, click, wait, verify, input, click, wait, verify, click, wait, verify, click, wait, wait_hidden, wait_hidden, wait, verify, wait_hidden, vision_compare_step, click, verify, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, wait, vision_compare_step, click, wait, vision_compare_step</t>
+          <t xml:space="preserve">set_viewport, click, wait, verify, input, click, wait, verify, click, wait, verify, click, wait, wait_hidden, wait_hidden, wait, verify, wait_hidden, wait, wait_hidden, verify, vision_compare_step, click, verify, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, vision_compare_step, click, wait, vision_compare_step, click, wait, vision_compare_step</t>
         </is>
       </c>
       <c r="J99" s="5" t="s">

</xml_diff>